<commit_message>
Added TestRunner and parallel run, multiple browser logic
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/opencarttestdata.xlsx
+++ b/src/test/resources/testdata/opencarttestdata.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5412F7E7-5F6A-4B5D-9C8C-95CA7102E6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{AA5131E8-DD5F-4717-AF8E-62A861746607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>